<commit_message>
feat: finalize tank class expansion baseline
</commit_message>
<xml_diff>
--- a/public/designer-data/challenge_encounter_balance.xlsx
+++ b/public/designer-data/challenge_encounter_balance.xlsx
@@ -130,10 +130,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -165,10 +165,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -596,7 +596,7 @@
         <v>100</v>
       </c>
       <c r="J4" t="str">
-        <v>8slot_0</v>
+        <v>standard_5slot</v>
       </c>
       <c r="K4" t="str">
         <v>1000</v>
@@ -649,7 +649,7 @@
         <v>100</v>
       </c>
       <c r="J5" t="str">
-        <v>standard_5slot</v>
+        <v>8slot_0</v>
       </c>
       <c r="K5" t="str">
         <v>1000</v>
@@ -702,7 +702,7 @@
         <v>100</v>
       </c>
       <c r="J6" t="str">
-        <v>standard_5slot</v>
+        <v>8slot_0</v>
       </c>
       <c r="K6" t="str">
         <v>1000</v>
@@ -808,7 +808,7 @@
         <v>95</v>
       </c>
       <c r="J8" t="str">
-        <v>standard_5slot</v>
+        <v>8slot_2</v>
       </c>
       <c r="K8">
         <v>1000</v>
@@ -861,7 +861,7 @@
         <v>105</v>
       </c>
       <c r="J9" t="str">
-        <v>8slot_0</v>
+        <v>8slot_2</v>
       </c>
       <c r="K9">
         <v>1000</v>
@@ -914,7 +914,7 @@
         <v>130</v>
       </c>
       <c r="J10" t="str">
-        <v>8slot_0</v>
+        <v>8slot_2</v>
       </c>
       <c r="K10">
         <v>1000</v>

</xml_diff>

<commit_message>
feat: add bear tank challenge balance loop
</commit_message>
<xml_diff>
--- a/public/designer-data/challenge_encounter_balance.xlsx
+++ b/public/designer-data/challenge_encounter_balance.xlsx
@@ -130,10 +130,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -165,10 +165,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -519,10 +519,10 @@
         <v>Challenge-2</v>
       </c>
       <c r="B3" t="str">
-        <v>120</v>
+        <v>140</v>
       </c>
       <c r="C3" t="str">
-        <v>120</v>
+        <v>140</v>
       </c>
       <c r="D3" t="str">
         <v>0</v>
@@ -561,7 +561,7 @@
         <v>4</v>
       </c>
       <c r="P3" t="str">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Q3" t="str">
         <v>0</v>
@@ -572,10 +572,10 @@
         <v>Challenge-3</v>
       </c>
       <c r="B4" t="str">
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="C4" t="str">
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="D4" t="str">
         <v>0</v>
@@ -614,7 +614,7 @@
         <v>4</v>
       </c>
       <c r="P4" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q4" t="str">
         <v>0</v>
@@ -1561,7 +1561,7 @@
         <v>Challenge-2-e03</v>
       </c>
       <c r="C9" t="str">
-        <v>murloc_blowgiller</v>
+        <v>murloc_tidehunter</v>
       </c>
       <c r="D9" t="str">
         <v>4</v>
@@ -1570,7 +1570,7 @@
         <v>2</v>
       </c>
       <c r="F9" t="str">
-        <v>鱼人吹箭者</v>
+        <v>鱼人猎潮者</v>
       </c>
       <c r="G9" t="str">
         <v/>
@@ -1751,7 +1751,7 @@
         <v>Challenge-3-e03</v>
       </c>
       <c r="C14" t="str">
-        <v>coldlight_seer</v>
+        <v>murloc_tidehunter</v>
       </c>
       <c r="D14" t="str">
         <v>3</v>
@@ -1760,7 +1760,7 @@
         <v>2</v>
       </c>
       <c r="F14" t="str">
-        <v>寒光先知</v>
+        <v>鱼人猎潮者</v>
       </c>
       <c r="G14" t="str">
         <v/>
@@ -3197,7 +3197,7 @@
         <v>dislike_affix_pic</v>
       </c>
       <c r="D2" t="str">
-        <v>你的队伍开场的三次攻击会产生5倍仇恨</v>
+        <v>你的队伍开场的三次攻击会产生2倍仇恨</v>
       </c>
       <c r="E2" t="str">
         <v>0</v>
@@ -3224,7 +3224,7 @@
         <v>3</v>
       </c>
       <c r="M2" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N2" t="str">
         <v/>

</xml_diff>

<commit_message>
balance: stabilize bear tank trial challenges
</commit_message>
<xml_diff>
--- a/public/designer-data/challenge_encounter_balance.xlsx
+++ b/public/designer-data/challenge_encounter_balance.xlsx
@@ -130,10 +130,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -165,10 +165,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -1307,10 +1307,10 @@
         <v>鱼人斥候</v>
       </c>
       <c r="G2" t="str">
-        <v/>
+        <v>80</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>80</v>
       </c>
       <c r="I2" t="str">
         <v>2</v>
@@ -1345,10 +1345,10 @@
         <v>鱼人斥候</v>
       </c>
       <c r="G3" t="str">
-        <v/>
+        <v>80</v>
       </c>
       <c r="H3" t="str">
-        <v/>
+        <v>80</v>
       </c>
       <c r="I3" t="str">
         <v>2</v>
@@ -1383,10 +1383,10 @@
         <v>鱼人猎潮者</v>
       </c>
       <c r="G4" t="str">
-        <v/>
+        <v>120</v>
       </c>
       <c r="H4" t="str">
-        <v/>
+        <v>120</v>
       </c>
       <c r="I4" t="str">
         <v>1</v>
@@ -1421,10 +1421,10 @@
         <v>鱼人吹箭者</v>
       </c>
       <c r="G5" t="str">
-        <v/>
+        <v>120</v>
       </c>
       <c r="H5" t="str">
-        <v/>
+        <v>120</v>
       </c>
       <c r="I5" t="str">
         <v>1</v>
@@ -1459,10 +1459,10 @@
         <v>寒光先知</v>
       </c>
       <c r="G6" t="str">
-        <v/>
+        <v>160</v>
       </c>
       <c r="H6" t="str">
-        <v/>
+        <v>160</v>
       </c>
       <c r="I6" t="str">
         <v>1</v>
@@ -1485,7 +1485,7 @@
         <v>Challenge-2-e01</v>
       </c>
       <c r="C7" t="str">
-        <v>kobold_monk</v>
+        <v>kobold_miner</v>
       </c>
       <c r="D7" t="str">
         <v>2</v>
@@ -1494,7 +1494,7 @@
         <v>2</v>
       </c>
       <c r="F7" t="str">
-        <v>狗头人武僧</v>
+        <v>狗头人矿工</v>
       </c>
       <c r="G7" t="str">
         <v/>
@@ -1789,7 +1789,7 @@
         <v>Challenge-3-e04</v>
       </c>
       <c r="C15" t="str">
-        <v>coldlight_oracle</v>
+        <v>murloc_tidehunter</v>
       </c>
       <c r="D15" t="str">
         <v>2</v>
@@ -1798,7 +1798,7 @@
         <v>3</v>
       </c>
       <c r="F15" t="str">
-        <v>寒光智者</v>
+        <v>鱼人猎潮者</v>
       </c>
       <c r="G15" t="str">
         <v/>

</xml_diff>

<commit_message>
feat: complete bear tank balance baseline
</commit_message>
<xml_diff>
--- a/public/designer-data/challenge_encounter_balance.xlsx
+++ b/public/designer-data/challenge_encounter_balance.xlsx
@@ -130,10 +130,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -165,10 +165,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -561,7 +561,7 @@
         <v>4</v>
       </c>
       <c r="P3" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q3" t="str">
         <v>0</v>
@@ -1789,7 +1789,7 @@
         <v>Challenge-3-e04</v>
       </c>
       <c r="C15" t="str">
-        <v>murloc_tidehunter</v>
+        <v>coldlight_seer</v>
       </c>
       <c r="D15" t="str">
         <v>2</v>
@@ -1798,7 +1798,7 @@
         <v>3</v>
       </c>
       <c r="F15" t="str">
-        <v>鱼人猎潮者</v>
+        <v>寒光先知</v>
       </c>
       <c r="G15" t="str">
         <v/>
@@ -2066,11 +2066,11 @@
       <c r="F22" t="str">
         <v>寒光先知</v>
       </c>
-      <c r="G22" t="str">
-        <v/>
-      </c>
-      <c r="H22" t="str">
-        <v/>
+      <c r="G22">
+        <v>550</v>
+      </c>
+      <c r="H22">
+        <v>550</v>
       </c>
       <c r="I22" t="str">
         <v>1</v>
@@ -2104,11 +2104,11 @@
       <c r="F23" t="str">
         <v>寒光智者</v>
       </c>
-      <c r="G23" t="str">
-        <v/>
-      </c>
-      <c r="H23" t="str">
-        <v/>
+      <c r="G23">
+        <v>825</v>
+      </c>
+      <c r="H23">
+        <v>825</v>
       </c>
       <c r="I23" t="str">
         <v>1</v>
@@ -3352,7 +3352,7 @@
       <c r="K5" t="str">
         <v>TRUE</v>
       </c>
-      <c r="L5" t="str">
+      <c r="L5">
         <v>55</v>
       </c>
       <c r="M5" t="str">
@@ -3461,7 +3461,7 @@
         <v>challenge_tide_order</v>
       </c>
       <c r="D8" t="str">
-        <v>后排或鱼人单位成功造成伤害时，对目标施加潮汐破绽：受到伤害提高10%，至多5层。</v>
+        <v>后排或鱼人单位成功造成伤害时，对目标施加潮汐破绽：受到伤害提高18%，至多5层。</v>
       </c>
       <c r="E8" t="str">
         <v>0</v>
@@ -3485,7 +3485,7 @@
         <v>TRUE</v>
       </c>
       <c r="L8">
-        <v>0.1</v>
+        <v>0.18</v>
       </c>
       <c r="M8">
         <v>5</v>

</xml_diff>